<commit_message>
tamaño de las pantallas, carteles, editar y borrar de todas las clases sin tener que ingresar id, ingresar el pedido mediante un desplegable
</commit_message>
<xml_diff>
--- a/data/db/pizzeria.xlsx
+++ b/data/db/pizzeria.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="97">
   <si>
     <t>ID</t>
   </si>
@@ -46,54 +46,51 @@
     <t>hola</t>
   </si>
   <si>
-    <t>ENTREGADA</t>
+    <t>PEDIDA</t>
   </si>
   <si>
     <t>2024-11-18 13:00:30.7411</t>
   </si>
   <si>
-    <t>20</t>
+    <t>15</t>
+  </si>
+  <si>
+    <t>TAMARA</t>
+  </si>
+  <si>
+    <t>editando</t>
+  </si>
+  <si>
+    <t>6000.0</t>
+  </si>
+  <si>
+    <t>142</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2024-11-21 13:18:52.2748</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Agua</t>
+  </si>
+  <si>
+    <t>1800.0</t>
+  </si>
+  <si>
+    <t>143</t>
+  </si>
+  <si>
+    <t>2024-11-22 15:32:48.542912</t>
   </si>
   <si>
     <t>MIRIAM</t>
   </si>
   <si>
-    <t>editando</t>
-  </si>
-  <si>
-    <t>6000.0</t>
-  </si>
-  <si>
-    <t>142</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>PEDIDA</t>
-  </si>
-  <si>
-    <t>2024-11-21 13:18:52.2748</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>TAMARA</t>
-  </si>
-  <si>
-    <t>Agua</t>
-  </si>
-  <si>
-    <t>1800.0</t>
-  </si>
-  <si>
-    <t>143</t>
-  </si>
-  <si>
-    <t>2024-11-22 15:32:48.542912</t>
-  </si>
-  <si>
     <t>pedido generado</t>
   </si>
   <si>
@@ -118,52 +115,73 @@
     <t>145</t>
   </si>
   <si>
+    <t>2024-11-23 17:43:52.867614</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>categoria: pasta : 3 Tallarines; categoria: salsa : 3 Salsa Fileto</t>
+  </si>
+  <si>
+    <t>9600.0</t>
+  </si>
+  <si>
+    <t>146</t>
+  </si>
+  <si>
+    <t>PREPARADA</t>
+  </si>
+  <si>
+    <t>2024-11-23 17:47:05.39782</t>
+  </si>
+  <si>
+    <t>69</t>
+  </si>
+  <si>
+    <t>1 pizza: Napolitana Especial; 2 faina: Faina; 3 gaseosa: Agua mineral; 2 cerveza: Andes IPA LATA</t>
+  </si>
+  <si>
+    <t>96600.0</t>
+  </si>
+  <si>
+    <t>148</t>
+  </si>
+  <si>
     <t>EN_PROCESO</t>
   </si>
   <si>
-    <t>2024-11-23 17:43:52.867614</t>
-  </si>
-  <si>
-    <t>MANUELA</t>
-  </si>
-  <si>
-    <t>4 pizza: Jamon</t>
-  </si>
-  <si>
-    <t>9600.0</t>
-  </si>
-  <si>
-    <t>146</t>
-  </si>
-  <si>
-    <t>PREPARADA</t>
-  </si>
-  <si>
-    <t>2024-11-23 17:47:05.39782</t>
-  </si>
-  <si>
-    <t>69</t>
-  </si>
-  <si>
-    <t>1 pizza: Napolitana Especial; 2 faina: Faina; 3 gaseosa: Agua mineral; 2 cerveza: Andes IPA LATA</t>
-  </si>
-  <si>
-    <t>96600.0</t>
-  </si>
-  <si>
-    <t>147</t>
-  </si>
-  <si>
-    <t>2024-11-23 17:51:37.465626</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>categoria: pizza : 3 Napolitana Especial; categoria: cerveza : 4 Andes IPA LATA</t>
-  </si>
-  <si>
-    <t>655.0</t>
+    <t>2024-11-25 17:01:12.244834</t>
+  </si>
+  <si>
+    <t>CAMILA</t>
+  </si>
+  <si>
+    <t>categoria: pizza : 3 Napolitana Especial; categoria: faina : 2 Faina; categoria: cerveza : 3 Stella Artois LATA</t>
+  </si>
+  <si>
+    <t>6500.0</t>
+  </si>
+  <si>
+    <t>149</t>
+  </si>
+  <si>
+    <t>2024-11-25 17:20:04.922713</t>
+  </si>
+  <si>
+    <t>categoria: pizza : 3 Napolitana Especial; categoria: gaseosa : 2 Gaseosas 1,5 lts</t>
+  </si>
+  <si>
+    <t>5600.0</t>
+  </si>
+  <si>
+    <t>181</t>
+  </si>
+  <si>
+    <t>2024-11-26 10:21:55.183961</t>
+  </si>
+  <si>
+    <t>categoria: guarniciones : 4 Pure de Calabaza</t>
   </si>
   <si>
     <t>DESCRIPCION</t>
@@ -181,6 +199,9 @@
     <t>35</t>
   </si>
   <si>
+    <t>editando compra 35</t>
+  </si>
+  <si>
     <t>2024-11-08 17:18:51.135972</t>
   </si>
   <si>
@@ -202,9 +223,6 @@
     <t>5466.0</t>
   </si>
   <si>
-    <t>CAMILA</t>
-  </si>
-  <si>
     <t>37</t>
   </si>
   <si>
@@ -214,9 +232,6 @@
     <t>2024-11-11 10:09:23.268909</t>
   </si>
   <si>
-    <t>5600.0</t>
-  </si>
-  <si>
     <t>41</t>
   </si>
   <si>
@@ -229,13 +244,67 @@
     <t>45600.0</t>
   </si>
   <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>un aceite,dos leches</t>
+  </si>
+  <si>
+    <t>2024-11-23 17:59:14.175846</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>aceite</t>
+  </si>
+  <si>
+    <t>2024-11-25 17:04:12.438611</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>jamon</t>
+  </si>
+  <si>
+    <t>2024-11-25 17:42:51.723026</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>2024-11-26 10:25:41.513022</t>
+  </si>
+  <si>
     <t>6</t>
   </si>
   <si>
-    <t>venta del dia editada</t>
+    <t>editandooo</t>
   </si>
   <si>
     <t>2024-11-15 13:05:44.900928</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">venta del dia </t>
+  </si>
+  <si>
+    <t>2024-11-26 10:27:08.787139</t>
+  </si>
+  <si>
+    <t>300000.0</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>2024-11-26 10:27:40.180511</t>
+  </si>
+  <si>
+    <t>300000.65</t>
   </si>
 </sst>
 </file>
@@ -280,7 +349,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -343,152 +412,204 @@
         <v>17</v>
       </c>
       <c r="C3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="E3" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="F3" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="F3" t="s" s="0">
+      <c r="H3" t="s" s="0">
         <v>21</v>
-      </c>
-      <c r="G3" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s" s="0">
         <v>17</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="E4" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="G4" t="s" s="0">
+      <c r="H4" t="s" s="0">
         <v>26</v>
-      </c>
-      <c r="H4" t="s" s="0">
-        <v>27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s" s="0">
         <v>17</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="E5" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="F5" t="s" s="0">
+      <c r="G5" t="s" s="0">
         <v>30</v>
       </c>
-      <c r="G5" t="s" s="0">
+      <c r="H5" t="s" s="0">
         <v>31</v>
-      </c>
-      <c r="H5" t="s" s="0">
-        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>17</v>
       </c>
       <c r="C6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="D6" t="s" s="0">
+      <c r="F6" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="G6" t="s" s="0">
         <v>35</v>
       </c>
-      <c r="E6" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="F6" t="s" s="0">
+      <c r="H6" t="s" s="0">
         <v>36</v>
-      </c>
-      <c r="G6" t="s" s="0">
-        <v>37</v>
-      </c>
-      <c r="H6" t="s" s="0">
-        <v>38</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s" s="0">
         <v>17</v>
       </c>
       <c r="C7" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E7" t="s" s="0">
         <v>40</v>
       </c>
-      <c r="D7" t="s" s="0">
+      <c r="F7" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="G7" t="s" s="0">
         <v>41</v>
       </c>
-      <c r="E7" t="s" s="0">
+      <c r="H7" t="s" s="0">
         <v>42</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s" s="0">
-        <v>43</v>
-      </c>
-      <c r="H7" t="s" s="0">
-        <v>44</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s" s="0">
         <v>17</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="E8" t="s" s="0">
+      <c r="G8" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="F8" t="s" s="0">
+      <c r="H8" t="s" s="0">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="G8" t="s" s="0">
-        <v>48</v>
-      </c>
-      <c r="H8" t="s" s="0">
-        <v>49</v>
+      <c r="G10" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="H10" t="s" s="0">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -498,7 +619,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -506,84 +627,152 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>14</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>84</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -593,7 +782,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -601,27 +790,55 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>66</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>94</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>95</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>